<commit_message>
VWAP mensuel mis à jour
</commit_message>
<xml_diff>
--- a/Nexans_VWAP.xlsx
+++ b/Nexans_VWAP.xlsx
@@ -21,6 +21,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025-08" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-07" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-08" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-09" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -213,6 +214,23 @@
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="Table_202608" displayName="Table_202608" ref="A1:H22" headerRowCount="1">
   <autoFilter ref="A1:H22"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="Date"/>
+    <tableColumn id="2" name="Adj Close"/>
+    <tableColumn id="3" name="Close"/>
+    <tableColumn id="4" name="High"/>
+    <tableColumn id="5" name="Low"/>
+    <tableColumn id="6" name="Open"/>
+    <tableColumn id="7" name="Volume"/>
+    <tableColumn id="8" name="VWAP"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="Table_202609" displayName="Table_202609" ref="A1:H23" headerRowCount="1">
+  <autoFilter ref="A1:H23"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Date"/>
     <tableColumn id="2" name="Adj Close"/>
@@ -4432,13 +4450,644 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Adj Close</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Close</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Volume</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>VWAP</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B2" t="n">
+        <v>137.5</v>
+      </c>
+      <c r="C2" t="n">
+        <v>137.5</v>
+      </c>
+      <c r="D2" t="n">
+        <v>140.8000030517578</v>
+      </c>
+      <c r="E2" t="n">
+        <v>135.8999938964844</v>
+      </c>
+      <c r="F2" t="n">
+        <v>139</v>
+      </c>
+      <c r="G2" t="n">
+        <v>160561</v>
+      </c>
+      <c r="H2" t="n">
+        <v>137.5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B3" t="n">
+        <v>137.6999969482422</v>
+      </c>
+      <c r="C3" t="n">
+        <v>137.6999969482422</v>
+      </c>
+      <c r="D3" t="n">
+        <v>139.3000030517578</v>
+      </c>
+      <c r="E3" t="n">
+        <v>136.1999969482422</v>
+      </c>
+      <c r="F3" t="n">
+        <v>136.8000030517578</v>
+      </c>
+      <c r="G3" t="n">
+        <v>97666</v>
+      </c>
+      <c r="H3" t="n">
+        <v>137.5756423687183</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B4" t="n">
+        <v>138.6000061035156</v>
+      </c>
+      <c r="C4" t="n">
+        <v>138.6000061035156</v>
+      </c>
+      <c r="D4" t="n">
+        <v>140</v>
+      </c>
+      <c r="E4" t="n">
+        <v>137.1999969482422</v>
+      </c>
+      <c r="F4" t="n">
+        <v>137.6999969482422</v>
+      </c>
+      <c r="G4" t="n">
+        <v>85863</v>
+      </c>
+      <c r="H4" t="n">
+        <v>137.8312584672998</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B5" t="n">
+        <v>136.6000061035156</v>
+      </c>
+      <c r="C5" t="n">
+        <v>136.6000061035156</v>
+      </c>
+      <c r="D5" t="n">
+        <v>140.6999969482422</v>
+      </c>
+      <c r="E5" t="n">
+        <v>136.3000030517578</v>
+      </c>
+      <c r="F5" t="n">
+        <v>139.8000030517578</v>
+      </c>
+      <c r="G5" t="n">
+        <v>116914</v>
+      </c>
+      <c r="H5" t="n">
+        <v>137.5190038255625</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B6" t="n">
+        <v>138.6000061035156</v>
+      </c>
+      <c r="C6" t="n">
+        <v>138.6000061035156</v>
+      </c>
+      <c r="D6" t="n">
+        <v>139.8000030517578</v>
+      </c>
+      <c r="E6" t="n">
+        <v>137.3999938964844</v>
+      </c>
+      <c r="F6" t="n">
+        <v>137.3999938964844</v>
+      </c>
+      <c r="G6" t="n">
+        <v>67522</v>
+      </c>
+      <c r="H6" t="n">
+        <v>137.6571076006122</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B7" t="n">
+        <v>141.3000030517578</v>
+      </c>
+      <c r="C7" t="n">
+        <v>141.3000030517578</v>
+      </c>
+      <c r="D7" t="n">
+        <v>141.5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>137.8000030517578</v>
+      </c>
+      <c r="F7" t="n">
+        <v>138.1000061035156</v>
+      </c>
+      <c r="G7" t="n">
+        <v>90505</v>
+      </c>
+      <c r="H7" t="n">
+        <v>138.1897146151332</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B8" t="n">
+        <v>138.5</v>
+      </c>
+      <c r="C8" t="n">
+        <v>138.5</v>
+      </c>
+      <c r="D8" t="n">
+        <v>141.6999969482422</v>
+      </c>
+      <c r="E8" t="n">
+        <v>137.5</v>
+      </c>
+      <c r="F8" t="n">
+        <v>141</v>
+      </c>
+      <c r="G8" t="n">
+        <v>134616</v>
+      </c>
+      <c r="H8" t="n">
+        <v>138.2451376147195</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B9" t="n">
+        <v>139.1999969482422</v>
+      </c>
+      <c r="C9" t="n">
+        <v>139.1999969482422</v>
+      </c>
+      <c r="D9" t="n">
+        <v>143.3999938964844</v>
+      </c>
+      <c r="E9" t="n">
+        <v>137.6000061035156</v>
+      </c>
+      <c r="F9" t="n">
+        <v>138.1999969482422</v>
+      </c>
+      <c r="G9" t="n">
+        <v>210295</v>
+      </c>
+      <c r="H9" t="n">
+        <v>138.4534511268843</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B10" t="n">
+        <v>142.1999969482422</v>
+      </c>
+      <c r="C10" t="n">
+        <v>142.1999969482422</v>
+      </c>
+      <c r="D10" t="n">
+        <v>145.6000061035156</v>
+      </c>
+      <c r="E10" t="n">
+        <v>138.6000061035156</v>
+      </c>
+      <c r="F10" t="n">
+        <v>139.5</v>
+      </c>
+      <c r="G10" t="n">
+        <v>198069</v>
+      </c>
+      <c r="H10" t="n">
+        <v>139.0920634845045</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B11" t="n">
+        <v>131.3999938964844</v>
+      </c>
+      <c r="C11" t="n">
+        <v>131.3999938964844</v>
+      </c>
+      <c r="D11" t="n">
+        <v>140.5</v>
+      </c>
+      <c r="E11" t="n">
+        <v>131.1000061035156</v>
+      </c>
+      <c r="F11" t="n">
+        <v>140.3999938964844</v>
+      </c>
+      <c r="G11" t="n">
+        <v>210677</v>
+      </c>
+      <c r="H11" t="n">
+        <v>137.911502319407</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B12" t="n">
+        <v>133.3999938964844</v>
+      </c>
+      <c r="C12" t="n">
+        <v>133.3999938964844</v>
+      </c>
+      <c r="D12" t="n">
+        <v>133.8999938964844</v>
+      </c>
+      <c r="E12" t="n">
+        <v>130.8999938964844</v>
+      </c>
+      <c r="F12" t="n">
+        <v>132.3000030517578</v>
+      </c>
+      <c r="G12" t="n">
+        <v>142614</v>
+      </c>
+      <c r="H12" t="n">
+        <v>137.4868976780704</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B13" t="n">
+        <v>136.6000061035156</v>
+      </c>
+      <c r="C13" t="n">
+        <v>136.6000061035156</v>
+      </c>
+      <c r="D13" t="n">
+        <v>137</v>
+      </c>
+      <c r="E13" t="n">
+        <v>133.6999969482422</v>
+      </c>
+      <c r="F13" t="n">
+        <v>133.6999969482422</v>
+      </c>
+      <c r="G13" t="n">
+        <v>155844</v>
+      </c>
+      <c r="H13" t="n">
+        <v>137.4041899251003</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B14" t="n">
+        <v>138.3999938964844</v>
+      </c>
+      <c r="C14" t="n">
+        <v>138.3999938964844</v>
+      </c>
+      <c r="D14" t="n">
+        <v>139.1999969482422</v>
+      </c>
+      <c r="E14" t="n">
+        <v>135.8999938964844</v>
+      </c>
+      <c r="F14" t="n">
+        <v>137.1999969482422</v>
+      </c>
+      <c r="G14" t="n">
+        <v>128911</v>
+      </c>
+      <c r="H14" t="n">
+        <v>137.4755043811176</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B15" t="n">
+        <v>136.8000030517578</v>
+      </c>
+      <c r="C15" t="n">
+        <v>136.8000030517578</v>
+      </c>
+      <c r="D15" t="n">
+        <v>140</v>
+      </c>
+      <c r="E15" t="n">
+        <v>136.8000030517578</v>
+      </c>
+      <c r="F15" t="n">
+        <v>138.6999969482422</v>
+      </c>
+      <c r="G15" t="n">
+        <v>172579</v>
+      </c>
+      <c r="H15" t="n">
+        <v>137.4164071407146</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B16" t="n">
+        <v>140.8000030517578</v>
+      </c>
+      <c r="C16" t="n">
+        <v>140.8000030517578</v>
+      </c>
+      <c r="D16" t="n">
+        <v>141.1000061035156</v>
+      </c>
+      <c r="E16" t="n">
+        <v>138</v>
+      </c>
+      <c r="F16" t="n">
+        <v>138.3999938964844</v>
+      </c>
+      <c r="G16" t="n">
+        <v>110277</v>
+      </c>
+      <c r="H16" t="n">
+        <v>137.5955470309943</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B17" t="n">
+        <v>143.5</v>
+      </c>
+      <c r="C17" t="n">
+        <v>143.5</v>
+      </c>
+      <c r="D17" t="n">
+        <v>144.1000061035156</v>
+      </c>
+      <c r="E17" t="n">
+        <v>140.6999969482422</v>
+      </c>
+      <c r="F17" t="n">
+        <v>141</v>
+      </c>
+      <c r="G17" t="n">
+        <v>110484</v>
+      </c>
+      <c r="H17" t="n">
+        <v>137.8929613074922</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B18" t="n">
+        <v>141</v>
+      </c>
+      <c r="C18" t="n">
+        <v>141</v>
+      </c>
+      <c r="D18" t="n">
+        <v>144.3000030517578</v>
+      </c>
+      <c r="E18" t="n">
+        <v>140.8000030517578</v>
+      </c>
+      <c r="F18" t="n">
+        <v>143.8999938964844</v>
+      </c>
+      <c r="G18" t="n">
+        <v>89842</v>
+      </c>
+      <c r="H18" t="n">
+        <v>138.0152185789439</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B19" t="n">
+        <v>135.8999938964844</v>
+      </c>
+      <c r="C19" t="n">
+        <v>135.8999938964844</v>
+      </c>
+      <c r="D19" t="n">
+        <v>141</v>
+      </c>
+      <c r="E19" t="n">
+        <v>135.5</v>
+      </c>
+      <c r="F19" t="n">
+        <v>140.1000061035156</v>
+      </c>
+      <c r="G19" t="n">
+        <v>112299</v>
+      </c>
+      <c r="H19" t="n">
+        <v>137.9160602201053</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B20" t="n">
+        <v>135.6000061035156</v>
+      </c>
+      <c r="C20" t="n">
+        <v>135.6000061035156</v>
+      </c>
+      <c r="D20" t="n">
+        <v>139.1999969482422</v>
+      </c>
+      <c r="E20" t="n">
+        <v>135.6000061035156</v>
+      </c>
+      <c r="F20" t="n">
+        <v>137.3999938964844</v>
+      </c>
+      <c r="G20" t="n">
+        <v>92669</v>
+      </c>
+      <c r="H20" t="n">
+        <v>137.8298027588369</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B21" t="n">
+        <v>133.3999938964844</v>
+      </c>
+      <c r="C21" t="n">
+        <v>133.3999938964844</v>
+      </c>
+      <c r="D21" t="n">
+        <v>135.1000061035156</v>
+      </c>
+      <c r="E21" t="n">
+        <v>132.5</v>
+      </c>
+      <c r="F21" t="n">
+        <v>135</v>
+      </c>
+      <c r="G21" t="n">
+        <v>123219</v>
+      </c>
+      <c r="H21" t="n">
+        <v>137.6207841543617</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B22" t="n">
+        <v>133.1999969482422</v>
+      </c>
+      <c r="C22" t="n">
+        <v>133.1999969482422</v>
+      </c>
+      <c r="D22" t="n">
+        <v>135.5</v>
+      </c>
+      <c r="E22" t="n">
+        <v>131.8999938964844</v>
+      </c>
+      <c r="F22" t="n">
+        <v>134.3000030517578</v>
+      </c>
+      <c r="G22" t="n">
+        <v>133902</v>
+      </c>
+      <c r="H22" t="n">
+        <v>137.40516246964</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B23" t="n">
+        <v>131.8999938964844</v>
+      </c>
+      <c r="C23" t="n">
+        <v>131.8999938964844</v>
+      </c>
+      <c r="D23" t="n">
+        <v>135.3999938964844</v>
+      </c>
+      <c r="E23" t="n">
+        <v>131.8999938964844</v>
+      </c>
+      <c r="F23" t="n">
+        <v>133.8999938964844</v>
+      </c>
+      <c r="G23" t="n">
+        <v>168412</v>
+      </c>
+      <c r="H23" t="n">
+        <v>137.0869678298498</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4581,6 +5230,16 @@
       </c>
       <c r="B14" t="n">
         <v>138.6740203216475</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>137.0869678298498</v>
       </c>
     </row>
   </sheetData>

</xml_diff>